<commit_message>
Updated N fertiliser data
Adds N-content to Peas.
</commit_message>
<xml_diff>
--- a/data-preprocessing/rpc-footprints/1 - Crops/N fertiliser.xlsx
+++ b/data-preprocessing/rpc-footprints/1 - Crops/N fertiliser.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr filterPrivacy="1" updateLinks="never" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85629D09-B1AB-4161-A7B7-4BCA3CFCA6CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{916EBC08-63FA-4880-A697-77B5FD265A27}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="INFO" sheetId="117" r:id="rId1"/>
@@ -2689,7 +2689,7 @@
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="68">
+  <cellXfs count="64">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -2831,13 +2831,9 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="1" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="13">
     <cellStyle name="Hyperlink" xfId="11" xr:uid="{27B946F3-5790-4F7E-8391-6BBF48B2CC3B}"/>
@@ -3350,7 +3346,7 @@
   <cols>
     <col min="2" max="2" width="32.90625" customWidth="1"/>
     <col min="3" max="3" width="15.36328125" customWidth="1"/>
-    <col min="4" max="4" width="16.6328125" style="63" customWidth="1"/>
+    <col min="4" max="4" width="16.6328125" customWidth="1"/>
     <col min="5" max="175" width="5.6328125" customWidth="1"/>
     <col min="176" max="176" width="5.6328125" style="1" customWidth="1"/>
     <col min="177" max="202" width="5.6328125" customWidth="1"/>
@@ -3972,7 +3968,7 @@
       <c r="C5" s="22" t="s">
         <v>3</v>
       </c>
-      <c r="D5" s="64" t="s">
+      <c r="D5" s="26" t="s">
         <v>236</v>
       </c>
       <c r="E5" s="26" t="s">
@@ -4580,7 +4576,7 @@
       <c r="C6" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="D6" s="65">
+      <c r="D6" s="36">
         <f>0.9753*GL6+0.02473*AP6</f>
         <v>246.37218999999999</v>
       </c>
@@ -4629,7 +4625,7 @@
       <c r="C8" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="D8" s="63" t="s">
+      <c r="D8" t="s">
         <v>401</v>
       </c>
       <c r="BC8">
@@ -4649,7 +4645,7 @@
       <c r="C9" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="D9" s="63" t="s">
+      <c r="D9" t="s">
         <v>641</v>
       </c>
       <c r="FT9" s="56"/>
@@ -4664,7 +4660,7 @@
       <c r="C10" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="D10" s="63" t="s">
+      <c r="D10" t="s">
         <v>635</v>
       </c>
       <c r="BC10">
@@ -4682,7 +4678,7 @@
       <c r="C11" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="D11" s="63" t="s">
+      <c r="D11" t="s">
         <v>401</v>
       </c>
       <c r="BC11">
@@ -4722,7 +4718,7 @@
       <c r="C13" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="D13" s="65">
+      <c r="D13" s="36">
         <f>0.7067*CI13+0.1908*BG13+0.05134*AU13+0.05098*AQ13</f>
         <v>147.54371239</v>
       </c>
@@ -4752,7 +4748,7 @@
       <c r="C14" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="D14" s="63" t="s">
+      <c r="D14" t="s">
         <v>401</v>
       </c>
       <c r="BC14">
@@ -4772,7 +4768,7 @@
       <c r="C15" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="D15" s="63" t="s">
+      <c r="D15" t="s">
         <v>401</v>
       </c>
       <c r="BC15">
@@ -4792,7 +4788,7 @@
       <c r="C16" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="D16" s="63" t="s">
+      <c r="D16" t="s">
         <v>401</v>
       </c>
       <c r="AB16" s="19"/>
@@ -4813,7 +4809,7 @@
       <c r="C17" s="2" t="s">
         <v>125</v>
       </c>
-      <c r="D17" s="63" t="s">
+      <c r="D17" t="s">
         <v>401</v>
       </c>
       <c r="BC17">
@@ -4833,7 +4829,7 @@
       <c r="C18" s="2" t="s">
         <v>127</v>
       </c>
-      <c r="D18" s="63" t="s">
+      <c r="D18" t="s">
         <v>636</v>
       </c>
       <c r="BC18">
@@ -4851,7 +4847,7 @@
       <c r="C19" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="D19" s="63" t="s">
+      <c r="D19" t="s">
         <v>627</v>
       </c>
       <c r="FT19" s="56"/>
@@ -4866,7 +4862,7 @@
       <c r="C20" s="2" t="s">
         <v>130</v>
       </c>
-      <c r="D20" s="63" t="s">
+      <c r="D20" t="s">
         <v>401</v>
       </c>
       <c r="BC20">
@@ -4904,7 +4900,7 @@
       <c r="C22" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="D22" s="63" t="s">
+      <c r="D22" t="s">
         <v>401</v>
       </c>
       <c r="BC22">
@@ -4924,7 +4920,7 @@
       <c r="C23" s="2" t="s">
         <v>134</v>
       </c>
-      <c r="D23" s="63" t="s">
+      <c r="D23" t="s">
         <v>645</v>
       </c>
     </row>
@@ -4938,7 +4934,7 @@
       <c r="C24" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="D24" s="63" t="s">
+      <c r="D24" t="s">
         <v>401</v>
       </c>
       <c r="BC24">
@@ -4958,7 +4954,7 @@
       <c r="C25" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="D25" s="63" t="s">
+      <c r="D25" t="s">
         <v>397</v>
       </c>
       <c r="FP25">
@@ -4975,7 +4971,7 @@
       <c r="C26" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="D26" s="63" t="s">
+      <c r="D26" t="s">
         <v>401</v>
       </c>
       <c r="BC26">
@@ -4995,7 +4991,7 @@
       <c r="C27" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="D27" s="63" t="s">
+      <c r="D27" t="s">
         <v>312</v>
       </c>
       <c r="CI27">
@@ -5051,7 +5047,7 @@
       <c r="C30" s="2" t="s">
         <v>127</v>
       </c>
-      <c r="D30" s="63" t="s">
+      <c r="D30" t="s">
         <v>636</v>
       </c>
       <c r="M30" s="28"/>
@@ -5067,7 +5063,7 @@
       <c r="C31" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="D31" s="63" t="s">
+      <c r="D31" t="s">
         <v>627</v>
       </c>
       <c r="FT31" s="57"/>
@@ -5097,7 +5093,7 @@
       <c r="C33" s="2" t="s">
         <v>145</v>
       </c>
-      <c r="D33" s="63" t="s">
+      <c r="D33" t="s">
         <v>397</v>
       </c>
       <c r="FP33">
@@ -5115,7 +5111,7 @@
       <c r="C34" s="2" t="s">
         <v>147</v>
       </c>
-      <c r="D34" s="65">
+      <c r="D34" s="36">
         <f>0.478*AZ34+0.269*CJ34+0.253*BX34</f>
         <v>32.094000000000001</v>
       </c>
@@ -5140,7 +5136,7 @@
       <c r="C35" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="D35" s="65">
+      <c r="D35" s="36">
         <f>0.4136*CJ35+0.3486*EO35+0.2379*CI35</f>
         <v>100.37289237499999</v>
       </c>
@@ -5168,7 +5164,7 @@
       <c r="C36" s="2" t="s">
         <v>147</v>
       </c>
-      <c r="D36" s="65">
+      <c r="D36" s="36">
         <f>0.4429*GQ36+0.2477*AA36+0.2386*CJ36+0.07079*CI36</f>
         <v>469.83887000000004</v>
       </c>
@@ -5199,7 +5195,7 @@
       <c r="C37" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="D37" s="63" t="s">
+      <c r="D37" t="s">
         <v>401</v>
       </c>
       <c r="BC37">
@@ -5219,7 +5215,7 @@
       <c r="C38" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="D38" s="63" t="s">
+      <c r="D38" t="s">
         <v>401</v>
       </c>
       <c r="BC38">
@@ -5239,7 +5235,7 @@
       <c r="C39" s="2" t="s">
         <v>127</v>
       </c>
-      <c r="D39" s="63" t="s">
+      <c r="D39" t="s">
         <v>401</v>
       </c>
       <c r="BC39">
@@ -5259,7 +5255,7 @@
       <c r="C40" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="D40" s="63" t="s">
+      <c r="D40" t="s">
         <v>708</v>
       </c>
       <c r="FT40" s="57"/>
@@ -5274,7 +5270,7 @@
       <c r="C41" s="2" t="s">
         <v>155</v>
       </c>
-      <c r="D41" s="63" t="s">
+      <c r="D41" t="s">
         <v>638</v>
       </c>
       <c r="BC41">
@@ -5292,7 +5288,7 @@
       <c r="C42" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="D42" s="63" t="s">
+      <c r="D42" t="s">
         <v>635</v>
       </c>
       <c r="FT42" s="57"/>
@@ -5307,7 +5303,7 @@
       <c r="C43" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="D43" s="63" t="s">
+      <c r="D43" t="s">
         <v>641</v>
       </c>
       <c r="FT43" s="57"/>
@@ -5322,7 +5318,7 @@
       <c r="C44" s="2" t="s">
         <v>127</v>
       </c>
-      <c r="D44" s="63" t="s">
+      <c r="D44" t="s">
         <v>636</v>
       </c>
       <c r="FT44" s="57"/>
@@ -5354,7 +5350,7 @@
       <c r="C46" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="D46" s="63" t="s">
+      <c r="D46" t="s">
         <v>646</v>
       </c>
       <c r="FT46" s="57"/>
@@ -5369,7 +5365,7 @@
       <c r="C47" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="D47" s="63" t="s">
+      <c r="D47" t="s">
         <v>639</v>
       </c>
       <c r="FT47" s="57">
@@ -5386,7 +5382,7 @@
       <c r="C48" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="D48" s="66">
+      <c r="D48" s="63">
         <f>0.6941*AP48+0.2774*CI48+0.02849*J48</f>
         <v>72.171999999999997</v>
       </c>
@@ -5411,7 +5407,7 @@
       <c r="C49" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="D49" s="63" t="s">
+      <c r="D49" t="s">
         <v>627</v>
       </c>
       <c r="FT49" s="57"/>
@@ -5426,7 +5422,7 @@
       <c r="C50" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="D50" s="63" t="s">
+      <c r="D50" t="s">
         <v>318</v>
       </c>
       <c r="CO50" s="36">
@@ -5448,7 +5444,7 @@
       <c r="C51" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="D51" s="63" t="s">
+      <c r="D51" t="s">
         <v>401</v>
       </c>
       <c r="BC51">
@@ -5468,7 +5464,7 @@
       <c r="C52" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="D52" s="63" t="s">
+      <c r="D52" t="s">
         <v>397</v>
       </c>
       <c r="FP52">
@@ -5486,7 +5482,7 @@
       <c r="C53" s="2" t="s">
         <v>125</v>
       </c>
-      <c r="D53" s="63" t="s">
+      <c r="D53" t="s">
         <v>401</v>
       </c>
       <c r="FT53" s="57">
@@ -5503,7 +5499,7 @@
       <c r="C54" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="D54" s="63" t="s">
+      <c r="D54" t="s">
         <v>401</v>
       </c>
       <c r="BC54">
@@ -5523,7 +5519,7 @@
       <c r="C55" s="2" t="s">
         <v>134</v>
       </c>
-      <c r="D55" s="63" t="s">
+      <c r="D55" t="s">
         <v>401</v>
       </c>
       <c r="FP55">
@@ -5543,7 +5539,7 @@
       <c r="C56" s="2" t="s">
         <v>125</v>
       </c>
-      <c r="D56" s="63" t="s">
+      <c r="D56" t="s">
         <v>632</v>
       </c>
       <c r="BC56">
@@ -5561,7 +5557,7 @@
       <c r="C57" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="D57" s="63" t="s">
+      <c r="D57" t="s">
         <v>401</v>
       </c>
       <c r="BC57">
@@ -5620,7 +5616,7 @@
       <c r="C60" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="D60" s="63" t="s">
+      <c r="D60" t="s">
         <v>401</v>
       </c>
       <c r="BC60">
@@ -5640,7 +5636,7 @@
       <c r="C61" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="D61" s="67" t="s">
+      <c r="D61" s="2" t="s">
         <v>313</v>
       </c>
       <c r="CJ61">
@@ -5661,7 +5657,7 @@
       <c r="C62" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="D62" s="65">
+      <c r="D62" s="36">
         <f>0.6712*FP62+0.3288*CO62</f>
         <v>74.023319999999998</v>
       </c>
@@ -5684,7 +5680,7 @@
       <c r="C63" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="D63" s="63" t="s">
+      <c r="D63" t="s">
         <v>401</v>
       </c>
       <c r="BC63">
@@ -5722,7 +5718,7 @@
       <c r="C65" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="D65" s="63" t="s">
+      <c r="D65" t="s">
         <v>629</v>
       </c>
       <c r="BC65">
@@ -5742,7 +5738,7 @@
       <c r="C66" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="D66" s="63" t="s">
+      <c r="D66" t="s">
         <v>634</v>
       </c>
       <c r="BC66">
@@ -5760,7 +5756,7 @@
       <c r="C67" s="2" t="s">
         <v>185</v>
       </c>
-      <c r="D67" s="63" t="s">
+      <c r="D67" t="s">
         <v>640</v>
       </c>
       <c r="BC67">
@@ -5778,7 +5774,7 @@
       <c r="C68" s="2" t="s">
         <v>125</v>
       </c>
-      <c r="D68" s="63" t="s">
+      <c r="D68" t="s">
         <v>628</v>
       </c>
       <c r="BC68">
@@ -5798,7 +5794,7 @@
       <c r="C69" s="2" t="s">
         <v>147</v>
       </c>
-      <c r="D69" s="63" t="s">
+      <c r="D69" t="s">
         <v>734</v>
       </c>
       <c r="FT69" s="56"/>
@@ -5813,7 +5809,7 @@
       <c r="C70" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="D70" s="63" t="s">
+      <c r="D70" t="s">
         <v>635</v>
       </c>
       <c r="BC70">
@@ -5870,7 +5866,7 @@
       <c r="C73" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="D73" s="63" t="s">
+      <c r="D73" t="s">
         <v>401</v>
       </c>
       <c r="BC73">
@@ -5890,7 +5886,7 @@
       <c r="C74" s="2" t="s">
         <v>130</v>
       </c>
-      <c r="D74" s="63" t="s">
+      <c r="D74" t="s">
         <v>401</v>
       </c>
       <c r="BC74">
@@ -5910,7 +5906,7 @@
       <c r="C75" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="D75" s="63" t="s">
+      <c r="D75" t="s">
         <v>401</v>
       </c>
       <c r="BC75">
@@ -5930,7 +5926,7 @@
       <c r="C76" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="D76" s="67" t="s">
+      <c r="D76" s="2" t="s">
         <v>273</v>
       </c>
       <c r="AU76">
@@ -5949,7 +5945,7 @@
       <c r="C77" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="D77" s="63" t="s">
+      <c r="D77" t="s">
         <v>401</v>
       </c>
       <c r="FT77" s="56">
@@ -5966,7 +5962,7 @@
       <c r="C78" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="D78" s="63" t="s">
+      <c r="D78" t="s">
         <v>641</v>
       </c>
       <c r="FT78" s="56"/>
@@ -5996,7 +5992,7 @@
       <c r="C80" s="2" t="s">
         <v>155</v>
       </c>
-      <c r="D80" s="63" t="s">
+      <c r="D80" t="s">
         <v>401</v>
       </c>
       <c r="BC80">
@@ -6016,7 +6012,7 @@
       <c r="C81" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="D81" s="63" t="s">
+      <c r="D81" t="s">
         <v>401</v>
       </c>
       <c r="FT81" s="56">
@@ -6033,7 +6029,7 @@
       <c r="C82" s="2" t="s">
         <v>201</v>
       </c>
-      <c r="D82" s="63" t="s">
+      <c r="D82" t="s">
         <v>634</v>
       </c>
       <c r="FT82" s="56"/>
@@ -6063,7 +6059,7 @@
       <c r="C84" s="2" t="s">
         <v>185</v>
       </c>
-      <c r="D84" s="63" t="s">
+      <c r="D84" t="s">
         <v>401</v>
       </c>
       <c r="BC84">
@@ -6083,7 +6079,7 @@
       <c r="C85" s="2" t="s">
         <v>185</v>
       </c>
-      <c r="D85" s="63" t="s">
+      <c r="D85" t="s">
         <v>401</v>
       </c>
       <c r="BC85">
@@ -6103,7 +6099,7 @@
       <c r="C86" s="2" t="s">
         <v>185</v>
       </c>
-      <c r="D86" s="63" t="s">
+      <c r="D86" t="s">
         <v>401</v>
       </c>
       <c r="BC86">
@@ -6123,7 +6119,7 @@
       <c r="C87" s="2" t="s">
         <v>127</v>
       </c>
-      <c r="D87" s="63" t="s">
+      <c r="D87" t="s">
         <v>401</v>
       </c>
       <c r="FT87" s="56">
@@ -6196,7 +6192,7 @@
       <c r="C89" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="D89" s="63" t="s">
+      <c r="D89" t="s">
         <v>401</v>
       </c>
       <c r="BC89">
@@ -6259,7 +6255,7 @@
       <c r="C91" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="D91" s="63" t="s">
+      <c r="D91" t="s">
         <v>636</v>
       </c>
       <c r="BC91">
@@ -6331,7 +6327,7 @@
       <c r="C93" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="D93" s="63" t="s">
+      <c r="D93" t="s">
         <v>401</v>
       </c>
       <c r="BC93">
@@ -6351,7 +6347,7 @@
       <c r="C94" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="D94" s="63" t="s">
+      <c r="D94" t="s">
         <v>401</v>
       </c>
       <c r="BC94">
@@ -6371,7 +6367,7 @@
       <c r="C95" s="2" t="s">
         <v>215</v>
       </c>
-      <c r="D95" s="63" t="s">
+      <c r="D95" t="s">
         <v>401</v>
       </c>
       <c r="BC95">
@@ -6450,7 +6446,7 @@
       <c r="C98" s="2" t="s">
         <v>155</v>
       </c>
-      <c r="D98" s="63" t="s">
+      <c r="D98" t="s">
         <v>264</v>
       </c>
       <c r="AP98">
@@ -6468,7 +6464,7 @@
       <c r="C99" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="D99" s="63" t="s">
+      <c r="D99" t="s">
         <v>641</v>
       </c>
       <c r="FT99" s="56"/>
@@ -6483,7 +6479,7 @@
       <c r="C100" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="D100" s="63" t="s">
+      <c r="D100" t="s">
         <v>401</v>
       </c>
       <c r="BC100">
@@ -6503,7 +6499,7 @@
       <c r="C101" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="D101" s="63" t="s">
+      <c r="D101" t="s">
         <v>748</v>
       </c>
       <c r="BC101">
@@ -6521,7 +6517,7 @@
       <c r="C102" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="D102" s="63" t="s">
+      <c r="D102" t="s">
         <v>401</v>
       </c>
       <c r="BC102">
@@ -6541,7 +6537,7 @@
       <c r="C103" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="D103" s="63" t="s">
+      <c r="D103" t="s">
         <v>627</v>
       </c>
       <c r="FT103" s="56"/>
@@ -6556,7 +6552,7 @@
       <c r="C104" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="D104" s="63" t="s">
+      <c r="D104" t="s">
         <v>642</v>
       </c>
       <c r="FT104" s="56"/>
@@ -6571,7 +6567,7 @@
       <c r="C105" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="D105" s="63" t="s">
+      <c r="D105" t="s">
         <v>642</v>
       </c>
       <c r="FT105" s="56"/>
@@ -6586,7 +6582,7 @@
       <c r="C106" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="D106" s="63" t="s">
+      <c r="D106" t="s">
         <v>401</v>
       </c>
       <c r="BC106">
@@ -6606,7 +6602,7 @@
       <c r="C107" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="D107" s="63" t="s">
+      <c r="D107" t="s">
         <v>401</v>
       </c>
       <c r="BC107">
@@ -6626,7 +6622,7 @@
       <c r="C108" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="D108" s="63" t="s">
+      <c r="D108" t="s">
         <v>401</v>
       </c>
       <c r="BC108">
@@ -6696,11 +6692,11 @@
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
+      <c r="A3" s="37" t="s">
         <v>729</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="78.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:4" ht="31" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="25" t="s">
         <v>0</v>
       </c>
@@ -7457,6 +7453,10 @@
       <c r="C65" s="2" t="s">
         <v>111</v>
       </c>
+      <c r="D65">
+        <f>0.021/6.25</f>
+        <v>3.3600000000000001E-3</v>
+      </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A66" s="2" t="s">
@@ -7577,6 +7577,10 @@
       </c>
       <c r="C75" s="2" t="s">
         <v>111</v>
+      </c>
+      <c r="D75">
+        <f>0.021/6.25</f>
+        <v>3.3600000000000001E-3</v>
       </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.35">
@@ -7986,9 +7990,12 @@
       <c r="C115" s="2"/>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A3" r:id="rId1" xr:uid="{C879ADC7-81D3-4EBF-86D2-61BB228F73CB}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
-  <legacyDrawing r:id="rId2"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId2"/>
+  <legacyDrawing r:id="rId3"/>
 </worksheet>
 </file>
 
@@ -11538,23 +11545,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="20b5f8f8-e964-4ea5-9bc5-5fa83731a92f" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="dokument" ma:contentTypeID="0x010100A603BB68AE5C0F4C908E70EB4D1DDDC3" ma:contentTypeVersion="15" ma:contentTypeDescription="Skapa ett nytt dokument." ma:contentTypeScope="" ma:versionID="bc1901b771652496ef02f4cbdf878f9e">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="31ffec6e-e0c6-46d3-bf16-e7019fdf1f95" xmlns:ns4="20b5f8f8-e964-4ea5-9bc5-5fa83731a92f" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="6c61e44642a1e9e2aad865b2f0b39e8f" ns3:_="" ns4:_="">
     <xsd:import namespace="31ffec6e-e0c6-46d3-bf16-e7019fdf1f95"/>
@@ -11789,25 +11779,24 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A16A6EDB-4C6A-433C-9B54-BF88B9AEEE87}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="20b5f8f8-e964-4ea5-9bc5-5fa83731a92f" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{627ED23C-5EEB-4F10-AA20-79B788D8342E}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="20b5f8f8-e964-4ea5-9bc5-5fa83731a92f"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{27BF0A1B-B2BC-4159-BD4C-213AA0853490}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -11824,4 +11813,22 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{627ED23C-5EEB-4F10-AA20-79B788D8342E}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="20b5f8f8-e964-4ea5-9bc5-5fa83731a92f"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A16A6EDB-4C6A-433C-9B54-BF88B9AEEE87}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
New N fertiliser file
</commit_message>
<xml_diff>
--- a/data-preprocessing/rpc-footprints/1 - Crops/N fertiliser.xlsx
+++ b/data-preprocessing/rpc-footprints/1 - Crops/N fertiliser.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr filterPrivacy="1" updateLinks="never" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{916EBC08-63FA-4880-A697-77B5FD265A27}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46413638-2373-479F-89B1-85401360A5AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="INFO" sheetId="117" r:id="rId1"/>
@@ -123,7 +123,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2150" uniqueCount="751">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2160" uniqueCount="753">
   <si>
     <t>Crops</t>
   </si>
@@ -2466,6 +2466,12 @@
   </si>
   <si>
     <t>Approx cantaloupes</t>
+  </si>
+  <si>
+    <t>Yara (2018)</t>
+  </si>
+  <si>
+    <t>Yara (2018). Gödslingsråd. https://www.yara.se/contentassets/b2d039536ac14ce382a98e12dd92282e/yar0050_godslingsradet_2018_okt.pdf</t>
   </si>
 </sst>
 </file>
@@ -2689,7 +2695,7 @@
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="64">
+  <cellXfs count="66">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -2834,6 +2840,10 @@
     <xf numFmtId="1" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="1" fontId="22" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="22" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="13">
     <cellStyle name="Hyperlink" xfId="11" xr:uid="{27B946F3-5790-4F7E-8391-6BBF48B2CC3B}"/>
@@ -3341,7 +3351,7 @@
   <sheetPr>
     <tabColor theme="6" tint="0.59999389629810485"/>
   </sheetPr>
-  <dimension ref="A2:GT115"/>
+  <dimension ref="A2:GT118"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="32.90625" customWidth="1"/>
@@ -4888,7 +4898,10 @@
       <c r="BC21">
         <v>0</v>
       </c>
-      <c r="FT21" s="57"/>
+      <c r="FT21" s="64">
+        <f>AVERAGE(30,40)</f>
+        <v>35</v>
+      </c>
     </row>
     <row r="22" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A22" s="2" t="s">
@@ -4906,8 +4919,9 @@
       <c r="BC22">
         <v>215</v>
       </c>
-      <c r="FT22" s="57">
-        <v>150</v>
+      <c r="FT22" s="64">
+        <f>AVERAGE(180,250)</f>
+        <v>215</v>
       </c>
     </row>
     <row r="23" spans="1:176" x14ac:dyDescent="0.35">
@@ -4940,8 +4954,9 @@
       <c r="BC24">
         <v>285</v>
       </c>
-      <c r="FT24" s="56">
-        <v>200.00035800590709</v>
+      <c r="FT24" s="65">
+        <f>AVERAGE(180,300)</f>
+        <v>240</v>
       </c>
     </row>
     <row r="25" spans="1:176" x14ac:dyDescent="0.35">
@@ -4977,8 +4992,9 @@
       <c r="BC26">
         <v>400</v>
       </c>
-      <c r="FT26" s="57">
-        <v>83</v>
+      <c r="FT26" s="64">
+        <f>AVERAGE(60,150)</f>
+        <v>105</v>
       </c>
     </row>
     <row r="27" spans="1:176" x14ac:dyDescent="0.35">
@@ -5016,8 +5032,9 @@
         <v>255</v>
       </c>
       <c r="FP28" s="28"/>
-      <c r="FT28" s="57">
-        <v>220</v>
+      <c r="FT28" s="64">
+        <f>AVERAGE(220, 280)</f>
+        <v>250</v>
       </c>
     </row>
     <row r="29" spans="1:176" x14ac:dyDescent="0.35">
@@ -5033,8 +5050,9 @@
       <c r="D29" s="1" t="s">
         <v>401</v>
       </c>
-      <c r="FT29" s="56">
-        <v>192.00000000000003</v>
+      <c r="FT29" s="65">
+        <f>AVERAGE(FT28,FT22)</f>
+        <v>232.5</v>
       </c>
     </row>
     <row r="30" spans="1:176" x14ac:dyDescent="0.35">
@@ -5450,8 +5468,9 @@
       <c r="BC51">
         <v>225</v>
       </c>
-      <c r="FT51" s="57">
-        <v>219.9992474773388</v>
+      <c r="FT51" s="64">
+        <f>AVERAGE(180,220)</f>
+        <v>200</v>
       </c>
     </row>
     <row r="52" spans="1:176" x14ac:dyDescent="0.35">
@@ -5505,8 +5524,9 @@
       <c r="BC54">
         <v>150</v>
       </c>
-      <c r="FT54" s="57">
-        <v>103.99894409543754</v>
+      <c r="FT54" s="64">
+        <f>AVERAGE(100,150)</f>
+        <v>125</v>
       </c>
     </row>
     <row r="55" spans="1:176" x14ac:dyDescent="0.35">
@@ -5912,8 +5932,9 @@
       <c r="BC75">
         <v>0</v>
       </c>
-      <c r="FT75" s="56">
-        <v>0</v>
+      <c r="FT75" s="65">
+        <f>AVERAGE(30,40)</f>
+        <v>35</v>
       </c>
     </row>
     <row r="76" spans="1:176" x14ac:dyDescent="0.35">
@@ -6015,8 +6036,9 @@
       <c r="D81" t="s">
         <v>401</v>
       </c>
-      <c r="FT81" s="56">
-        <v>17.999882715781244</v>
+      <c r="FT81" s="65">
+        <f>AVERAGE(90,170)</f>
+        <v>130</v>
       </c>
     </row>
     <row r="82" spans="1:199" x14ac:dyDescent="0.35">
@@ -6652,20 +6674,23 @@
       <c r="B112" s="2"/>
       <c r="C112" s="2"/>
     </row>
-    <row r="113" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:181" x14ac:dyDescent="0.35">
       <c r="A113" s="2"/>
       <c r="B113" s="2"/>
       <c r="C113" s="2"/>
     </row>
-    <row r="114" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:181" x14ac:dyDescent="0.35">
       <c r="A114" s="2"/>
       <c r="B114" s="2"/>
       <c r="C114" s="2"/>
     </row>
-    <row r="115" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:181" x14ac:dyDescent="0.35">
       <c r="A115" s="2"/>
       <c r="B115" s="2"/>
       <c r="C115" s="2"/>
+    </row>
+    <row r="118" spans="1:181" x14ac:dyDescent="0.35">
+      <c r="FY118" s="19"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -9446,7 +9471,7 @@
         <v>676</v>
       </c>
     </row>
-    <row r="17" spans="1:172" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A17" s="2" t="s">
         <v>15</v>
       </c>
@@ -9466,7 +9491,7 @@
         <v>676</v>
       </c>
     </row>
-    <row r="18" spans="1:172" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A18" s="2" t="s">
         <v>16</v>
       </c>
@@ -9486,7 +9511,7 @@
         <v>676</v>
       </c>
     </row>
-    <row r="19" spans="1:172" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A19" s="2" t="s">
         <v>17</v>
       </c>
@@ -9502,7 +9527,7 @@
       <c r="BC19" s="44"/>
       <c r="BD19" s="44"/>
     </row>
-    <row r="20" spans="1:172" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A20" s="2" t="s">
         <v>18</v>
       </c>
@@ -9522,7 +9547,7 @@
         <v>679</v>
       </c>
     </row>
-    <row r="21" spans="1:172" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A21" s="2" t="s">
         <v>19</v>
       </c>
@@ -9541,8 +9566,11 @@
       <c r="BD21" s="41" t="s">
         <v>676</v>
       </c>
-    </row>
-    <row r="22" spans="1:172" x14ac:dyDescent="0.35">
+      <c r="FT21" t="s">
+        <v>751</v>
+      </c>
+    </row>
+    <row r="22" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A22" s="2" t="s">
         <v>20</v>
       </c>
@@ -9561,8 +9589,11 @@
       <c r="BD22" s="41" t="s">
         <v>676</v>
       </c>
-    </row>
-    <row r="23" spans="1:172" x14ac:dyDescent="0.35">
+      <c r="FT22" t="s">
+        <v>751</v>
+      </c>
+    </row>
+    <row r="23" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A23" s="2" t="s">
         <v>21</v>
       </c>
@@ -9578,7 +9609,7 @@
       <c r="BC23" s="44"/>
       <c r="BD23" s="44"/>
     </row>
-    <row r="24" spans="1:172" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A24" s="2" t="s">
         <v>22</v>
       </c>
@@ -9597,8 +9628,11 @@
       <c r="BD24" s="41" t="s">
         <v>676</v>
       </c>
-    </row>
-    <row r="25" spans="1:172" x14ac:dyDescent="0.35">
+      <c r="FT24" t="s">
+        <v>751</v>
+      </c>
+    </row>
+    <row r="25" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A25" s="2" t="s">
         <v>23</v>
       </c>
@@ -9617,7 +9651,7 @@
         <v>698</v>
       </c>
     </row>
-    <row r="26" spans="1:172" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A26" s="2" t="s">
         <v>24</v>
       </c>
@@ -9636,8 +9670,11 @@
       <c r="BD26" s="41" t="s">
         <v>676</v>
       </c>
-    </row>
-    <row r="27" spans="1:172" x14ac:dyDescent="0.35">
+      <c r="FT26" t="s">
+        <v>751</v>
+      </c>
+    </row>
+    <row r="27" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A27" s="2" t="s">
         <v>25</v>
       </c>
@@ -9656,7 +9693,7 @@
         <v>700</v>
       </c>
     </row>
-    <row r="28" spans="1:172" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A28" s="2" t="s">
         <v>26</v>
       </c>
@@ -9675,8 +9712,11 @@
       <c r="BD28" s="41" t="s">
         <v>676</v>
       </c>
-    </row>
-    <row r="29" spans="1:172" x14ac:dyDescent="0.35">
+      <c r="FT28" t="s">
+        <v>751</v>
+      </c>
+    </row>
+    <row r="29" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A29" s="2" t="s">
         <v>27</v>
       </c>
@@ -9692,7 +9732,7 @@
       <c r="BC29" s="39"/>
       <c r="BD29" s="39"/>
     </row>
-    <row r="30" spans="1:172" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A30" s="2" t="s">
         <v>28</v>
       </c>
@@ -9709,7 +9749,7 @@
       <c r="BC30" s="47"/>
       <c r="BD30" s="47"/>
     </row>
-    <row r="31" spans="1:172" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A31" s="2" t="s">
         <v>29</v>
       </c>
@@ -9725,7 +9765,7 @@
       <c r="BC31" s="47"/>
       <c r="BD31" s="47"/>
     </row>
-    <row r="32" spans="1:172" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A32" s="2" t="s">
         <v>30</v>
       </c>
@@ -10103,6 +10143,9 @@
       <c r="BD51" s="41" t="s">
         <v>676</v>
       </c>
+      <c r="FT51" t="s">
+        <v>751</v>
+      </c>
     </row>
     <row r="52" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A52" s="2" t="s">
@@ -10161,6 +10204,9 @@
       <c r="BD54" s="41" t="s">
         <v>676</v>
       </c>
+      <c r="FT54" t="s">
+        <v>751</v>
+      </c>
     </row>
     <row r="55" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A55" s="2" t="s">
@@ -10572,6 +10618,9 @@
       <c r="BD75" s="41" t="s">
         <v>676</v>
       </c>
+      <c r="FT75" t="s">
+        <v>751</v>
+      </c>
     </row>
     <row r="76" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A76" s="2" t="s">
@@ -10675,6 +10724,9 @@
       </c>
       <c r="BC81" s="39"/>
       <c r="BD81" s="39"/>
+      <c r="FT81" t="s">
+        <v>751</v>
+      </c>
     </row>
     <row r="82" spans="1:199" x14ac:dyDescent="0.35">
       <c r="A82" s="2" t="s">
@@ -11443,7 +11495,9 @@
       </c>
     </row>
     <row r="12" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A12" s="5"/>
+      <c r="A12" s="5" t="s">
+        <v>752</v>
+      </c>
       <c r="S12" s="9"/>
     </row>
     <row r="13" spans="1:22" x14ac:dyDescent="0.35">

</xml_diff>